<commit_message>
Cambios hechos en reto2
</commit_message>
<xml_diff>
--- a/database/06_REDES_CONEXIONES_SAN_MARTIN.xlsx
+++ b/database/06_REDES_CONEXIONES_SAN_MARTIN.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam Lenin\Desktop\DATATHON\CONCURSO\database\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF186542-497A-4B43-88E4-CE58752EEB0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="125725" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -315,8 +322,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -338,27 +345,365 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E85"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -375,7 +720,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -392,7 +737,7 @@
         <v>358.32829852593801</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -409,7 +754,7 @@
         <v>1963.6520189980199</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -426,7 +771,7 @@
         <v>968.21900550382099</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -443,7 +788,7 @@
         <v>2491.2697366134698</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -460,7 +805,7 @@
         <v>213.11476255313701</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -477,7 +822,7 @@
         <v>815.77763529352205</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -494,7 +839,7 @@
         <v>802.03620199710394</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -511,7 +856,7 @@
         <v>19.442641913185099</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -528,7 +873,7 @@
         <v>2408.5414078573899</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -545,7 +890,7 @@
         <v>275.35147824280699</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -562,7 +907,7 @@
         <v>21.843460185652798</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -579,7 +924,7 @@
         <v>861.50334480536901</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -596,7 +941,7 @@
         <v>720.17306683787501</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -613,7 +958,7 @@
         <v>513.37236795690603</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -630,7 +975,7 @@
         <v>644.29680722480396</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -647,7 +992,7 @@
         <v>11.694102935974399</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -664,7 +1009,7 @@
         <v>2611.3678496658899</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -681,7 +1026,7 @@
         <v>1439.82114402858</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -698,7 +1043,7 @@
         <v>216.197962315231</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -715,7 +1060,7 @@
         <v>3261.8218619593799</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -732,7 +1077,7 @@
         <v>2991.1131428191902</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -749,7 +1094,7 @@
         <v>382.197994809313</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -766,7 +1111,7 @@
         <v>2700.9789986128899</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -783,7 +1128,7 @@
         <v>490.34092327364402</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -800,7 +1145,7 @@
         <v>1989.2716391534</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -817,7 +1162,7 @@
         <v>3108.45297274109</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -834,7 +1179,7 @@
         <v>3469.0065556417799</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -851,7 +1196,7 @@
         <v>796.03261068162396</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -868,7 +1213,7 @@
         <v>1169.6301163184201</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -885,7 +1230,7 @@
         <v>118.93665860583199</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -902,7 +1247,7 @@
         <v>19.9896677060012</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -919,7 +1264,7 @@
         <v>1495.63824028717</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -936,7 +1281,7 @@
         <v>798.64643977250296</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -953,7 +1298,7 @@
         <v>2558.94006198334</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -970,7 +1315,7 @@
         <v>9388.5118419457103</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -987,7 +1332,7 @@
         <v>1164.82996253691</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -1004,7 +1349,7 @@
         <v>6005.7302577943901</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -1021,7 +1366,7 @@
         <v>2950.0435808852199</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -1038,7 +1383,7 @@
         <v>2984.9905599377398</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -1053,7 +1398,7 @@
       </c>
       <c r="E41" s="1"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -1070,7 +1415,7 @@
         <v>2212.6715519811601</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -1087,7 +1432,7 @@
         <v>5115.1592171000302</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -1104,7 +1449,7 @@
         <v>2759.7832909151998</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -1121,7 +1466,7 @@
         <v>3575.8127349441802</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -1138,7 +1483,7 @@
         <v>7088.0875689761197</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -1155,7 +1500,7 @@
         <v>2112.4015683970101</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -1172,7 +1517,7 @@
         <v>3095.5700694603202</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -1189,7 +1534,7 @@
         <v>3948.3343028272202</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -1206,7 +1551,7 @@
         <v>1265.90181649438</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -1223,7 +1568,7 @@
         <v>2938.8637110178602</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -1240,7 +1585,7 @@
         <v>1517.60829032877</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -1257,7 +1602,7 @@
         <v>10696.625564828</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -1274,7 +1619,7 @@
         <v>4203.8558932937503</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -1291,7 +1636,7 @@
         <v>613.18109372493598</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -1308,7 +1653,7 @@
         <v>3815.3747749120598</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -1325,7 +1670,7 @@
         <v>6162.5980388808903</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -1342,7 +1687,7 @@
         <v>1094.26813837645</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -1359,7 +1704,7 @@
         <v>2483.1569534844998</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -1376,7 +1721,7 @@
         <v>2023.14018065292</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -1393,7 +1738,7 @@
         <v>1828.3282149009599</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>61</v>
       </c>
@@ -1410,7 +1755,7 @@
         <v>5653.3079393358303</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>62</v>
       </c>
@@ -1427,7 +1772,7 @@
         <v>10086.840474971001</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -1444,7 +1789,7 @@
         <v>25.489181857469401</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>64</v>
       </c>
@@ -1461,7 +1806,7 @@
         <v>656.56980534853699</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>65</v>
       </c>
@@ -1478,7 +1823,7 @@
         <v>6056.5157891088202</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -1495,7 +1840,7 @@
         <v>1534.1481769843101</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -1512,7 +1857,7 @@
         <v>4544.00545811764</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -1529,7 +1874,7 @@
         <v>1.45320684613096</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -1546,7 +1891,7 @@
         <v>4043.9888666623901</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -1563,7 +1908,7 @@
         <v>7095.3178569957299</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -1580,7 +1925,7 @@
         <v>1912.47454972277</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -1597,7 +1942,7 @@
         <v>2413.32318705121</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -1614,7 +1959,7 @@
         <v>2153.5875505875701</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -1631,7 +1976,7 @@
         <v>9706.8646702319802</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -1648,7 +1993,7 @@
         <v>4754.77276241647</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -1665,7 +2010,7 @@
         <v>365.35603045118899</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -1682,7 +2027,7 @@
         <v>3895.60604127326</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -1699,7 +2044,7 @@
         <v>6554.3181462943303</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -1716,7 +2061,7 @@
         <v>3964.1513188265999</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>80</v>
       </c>
@@ -1733,7 +2078,7 @@
         <v>4587.5624000588896</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>81</v>
       </c>
@@ -1750,7 +2095,7 @@
         <v>3929.27833490376</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>82</v>
       </c>
@@ -1767,7 +2112,7 @@
         <v>5128.0850207081103</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -1784,7 +2129,7 @@
         <v>8274.7962586135509</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -1802,10 +2147,31 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a26aadba-2109-4707-979c-67af72fb5bed" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="81066592-8f5a-480f-93f4-ff267641d634">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006088ED23669E2B47B26706AE4D6E8B3B" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a0c8d670484223c018a903029ee63509">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="81066592-8f5a-480f-93f4-ff267641d634" xmlns:ns3="a26aadba-2109-4707-979c-67af72fb5bed" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="64572940cd0622e9cb3624eeb959aa1b" ns2:_="" ns3:_="">
     <xsd:import namespace="81066592-8f5a-480f-93f4-ff267641d634"/>
@@ -2046,34 +2412,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a26aadba-2109-4707-979c-67af72fb5bed" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="81066592-8f5a-480f-93f4-ff267641d634">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{296C6FB1-0C48-4B90-9BE0-0E2FB23AB029}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E96528-F153-4CE4-9BCB-1A5A39D3A46F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a26aadba-2109-4707-979c-67af72fb5bed"/>
+    <ds:schemaRef ds:uri="81066592-8f5a-480f-93f4-ff267641d634"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1E4C0FE-5B72-45E1-B485-37881748929E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C1E4C0FE-5B72-45E1-B485-37881748929E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00E96528-F153-4CE4-9BCB-1A5A39D3A46F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{296C6FB1-0C48-4B90-9BE0-0E2FB23AB029}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="81066592-8f5a-480f-93f4-ff267641d634"/>
+    <ds:schemaRef ds:uri="a26aadba-2109-4707-979c-67af72fb5bed"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>